<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 16:28 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4327.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4327.xlsx
@@ -218,9 +218,9 @@
     Planos para:
         Ventilador ZVN 2-9-103/2 con motor WEG o similar – Alcance: TOBERA + REJILLA + FAR 90/100 + VENT + FAR 90/100 + TIPO A
         Alcance Chile: TOBERA + REJILLA + VENT
-        Alcance Colombia: FAR + DIFUSOR
+        Alcance Colombia: FAR + TIPO A
     Rodete:
-        Ventilador ZVN 1-12-55/4 --- ALABES: 300004
+        Ventilador ZVN 2-9-103/2 --- ALABES: 300000
     Tratamiento superficial:
         Estándar Zitrón con 2 capas y color de terminación Blanco RAL 9001.
     Datos eléctricos para el motor:
@@ -232,79 +232,79 @@
     <t>Ingenieria Jefe de proyecto:,Analisis de costeo,Planos preliminar</t>
   </si>
   <si>
+    <t>1214977316716053</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
   </si>
   <si>
-    <t>1214977316716053</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
+    <t>1214969047720956</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta Corte Laser OT4327,propuesta motor OT4327,propuesta alabes OT4327,propuesta nucleo rodete OT4327</t>
+  </si>
+  <si>
+    <t>1214977316726320</t>
+  </si>
+  <si>
+    <t>propuesta motor OT4327</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT4327,Propuesta compras:</t>
+  </si>
+  <si>
+    <t>1214977316726340</t>
+  </si>
+  <si>
+    <t>propuesta alabes OT4327</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT4327,Propuesta compras:</t>
+  </si>
+  <si>
+    <t>1214977533910216</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete OT4327</t>
+  </si>
+  <si>
+    <t>benjamin.bustos@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete OT4327</t>
+  </si>
+  <si>
+    <t>1214977075717388</t>
+  </si>
+  <si>
+    <t>propuesta Corte Laser OT4327</t>
+  </si>
+  <si>
+    <t>hugo isla martinez</t>
+  </si>
+  <si>
+    <t>hugo.isla@zitron.com</t>
+  </si>
+  <si>
+    <t>check planos</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC materiales corte Laser OT4327</t>
   </si>
   <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214969047720956</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta Corte Laser OT4327,propuesta motor OT4327,propuesta alabes OT4327,propuesta nucleo rodete OT4327</t>
-  </si>
-  <si>
-    <t>1214977316726320</t>
-  </si>
-  <si>
-    <t>propuesta motor OT4327</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT4327,Propuesta compras:</t>
-  </si>
-  <si>
-    <t>1214977316726340</t>
-  </si>
-  <si>
-    <t>propuesta alabes OT4327</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT4327,Propuesta compras:</t>
-  </si>
-  <si>
-    <t>1214977533910216</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete OT4327</t>
-  </si>
-  <si>
-    <t>benjamin.bustos@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete OT4327</t>
-  </si>
-  <si>
-    <t>1214977075717388</t>
-  </si>
-  <si>
-    <t>propuesta Corte Laser OT4327</t>
-  </si>
-  <si>
-    <t>hugo isla martinez</t>
-  </si>
-  <si>
-    <t>hugo.isla@zitron.com</t>
-  </si>
-  <si>
-    <t>check planos</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC materiales corte Laser OT4327</t>
   </si>
   <si>
     <t>1214977075717403</t>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46197.669773472226</v>
+        <v>46197.67116355324</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -2643,9 +2643,11 @@
       <c r="B13" s="9">
         <v>46162.68130347222</v>
       </c>
-      <c r="C13" s="10"/>
+      <c r="C13" s="9">
+        <v>46197.671156689816</v>
+      </c>
       <c r="D13" s="9">
-        <v>46197.670623125</v>
+        <v>46197.671174166666</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>60</v>
@@ -2693,25 +2695,25 @@
         <v>54</v>
       </c>
       <c r="T13" s="10">
-        <v>0</v>
-      </c>
-      <c r="U13" s="12" t="s">
-        <v>63</v>
+        <v>1</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46162.6813085301</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46197.669773981484</v>
+        <v>46197.67117741898</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -2741,10 +2743,10 @@
         <v>46</v>
       </c>
       <c r="O14" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="P14" s="6" t="s">
         <v>66</v>
-      </c>
-      <c r="P14" s="6" t="s">
-        <v>67</v>
       </c>
       <c r="Q14" s="5">
         <v>46149</v>
@@ -2758,13 +2760,13 @@
       <c r="T14" s="6">
         <v>0</v>
       </c>
-      <c r="U14" s="11" t="s">
-        <v>68</v>
+      <c r="U14" s="12" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" s="9">
         <v>46162.68117188658</v>
@@ -2774,7 +2776,7 @@
         <v>46197.587885057874</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>25</v>
@@ -2798,7 +2800,7 @@
         <v>26</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>26</v>
@@ -2811,7 +2813,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46162.681316030095</v>
@@ -2821,7 +2823,7 @@
         <v>46197.66702332176</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2848,13 +2850,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>49</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Q16" s="5">
         <v>46153</v>
@@ -2869,12 +2871,12 @@
         <v>0</v>
       </c>
       <c r="U16" s="12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B17" s="9">
         <v>46162.68132108796</v>
@@ -2884,7 +2886,7 @@
         <v>46197.66978644676</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>26</v>
@@ -2911,13 +2913,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>56</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q17" s="9">
         <v>46153</v>
@@ -2932,12 +2934,12 @@
         <v>0</v>
       </c>
       <c r="U17" s="12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B18" s="5">
         <v>46162.68132700231</v>
@@ -2949,16 +2951,16 @@
         <v>46197.66978645833</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I18" s="5">
         <v>46153</v>
@@ -2976,13 +2978,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>56</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q18" s="5">
         <v>46153</v>
@@ -2997,12 +2999,12 @@
         <v>1</v>
       </c>
       <c r="U18" s="12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B19" s="9">
         <v>46162.68133263889</v>
@@ -3012,16 +3014,16 @@
         <v>46190.17346704861</v>
       </c>
       <c r="E19" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G19" s="10" t="s">
+      <c r="H19" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="I19" s="9">
         <v>46188</v>
@@ -3039,13 +3041,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O19" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="P19" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="P19" s="10" t="s">
-        <v>87</v>
       </c>
       <c r="Q19" s="9">
         <v>46188</v>
@@ -3060,7 +3062,7 @@
         <v>0</v>
       </c>
       <c r="U19" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -3081,10 +3083,10 @@
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="I20" s="5">
         <v>46184</v>
@@ -3102,10 +3104,10 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>90</v>
@@ -3123,7 +3125,7 @@
         <v>0</v>
       </c>
       <c r="U20" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
@@ -3144,10 +3146,10 @@
         <v>26</v>
       </c>
       <c r="G21" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="I21" s="9">
         <v>46188</v>
@@ -3165,10 +3167,10 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>93</v>
@@ -3186,7 +3188,7 @@
         <v>0</v>
       </c>
       <c r="U21" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
@@ -3207,10 +3209,10 @@
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="I22" s="5">
         <v>46188</v>
@@ -3228,10 +3230,10 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P22" s="6" t="s">
         <v>96</v>
@@ -3249,7 +3251,7 @@
         <v>0</v>
       </c>
       <c r="U22" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -3359,7 +3361,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -3404,7 +3406,7 @@
         <v>101</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>107</v>
@@ -3418,7 +3420,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -3477,7 +3479,7 @@
         <v>0</v>
       </c>
       <c r="U26" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -3540,7 +3542,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3585,7 +3587,7 @@
         <v>112</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>116</v>
@@ -3599,7 +3601,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3658,7 +3660,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3721,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3766,7 +3768,7 @@
         <v>121</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P31" s="10" t="s">
         <v>125</v>
@@ -3780,7 +3782,7 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3839,7 +3841,7 @@
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3898,7 +3900,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3961,7 +3963,7 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -4006,7 +4008,7 @@
         <v>133</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P35" s="10" t="s">
         <v>140</v>
@@ -4020,7 +4022,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -4075,7 +4077,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -4138,7 +4140,7 @@
         <v>0</v>
       </c>
       <c r="U37" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -4307,7 +4309,7 @@
         <v>0</v>
       </c>
       <c r="U40" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -4529,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="U44" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -4694,7 +4696,7 @@
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46168.16746090278</v>
+        <v>46197.671176655094</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>178</v>
@@ -4744,8 +4746,8 @@
       <c r="T48" s="6">
         <v>0</v>
       </c>
-      <c r="U48" s="11" t="s">
-        <v>68</v>
+      <c r="U48" s="12" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -4808,7 +4810,7 @@
         <v>0</v>
       </c>
       <c r="U49" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -4823,7 +4825,7 @@
         <v>46186.16887460648</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
@@ -4871,7 +4873,7 @@
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4932,7 +4934,7 @@
         <v>0</v>
       </c>
       <c r="U51" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -5550,7 +5552,7 @@
         <v>0</v>
       </c>
       <c r="U63" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -5611,7 +5613,7 @@
         <v>0</v>
       </c>
       <c r="U64" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5672,7 +5674,7 @@
         <v>0</v>
       </c>
       <c r="U65" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5733,7 +5735,7 @@
         <v>0</v>
       </c>
       <c r="U66" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5794,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="U67" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5855,7 +5857,7 @@
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5965,7 +5967,7 @@
         <v>0</v>
       </c>
       <c r="U70" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -6558,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="U81" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -7151,7 +7153,7 @@
         <v>0</v>
       </c>
       <c r="U92" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -7789,7 +7791,7 @@
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7850,7 +7852,7 @@
         <v>0</v>
       </c>
       <c r="U105" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
@@ -7911,7 +7913,7 @@
         <v>0</v>
       </c>
       <c r="U106" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
@@ -7972,7 +7974,7 @@
         <v>0</v>
       </c>
       <c r="U107" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
@@ -8040,10 +8042,10 @@
         <v>26</v>
       </c>
       <c r="G109" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H109" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I109" s="9">
         <v>46218</v>
@@ -8082,7 +8084,7 @@
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -8103,10 +8105,10 @@
         <v>26</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I110" s="5">
         <v>46218</v>
@@ -8156,10 +8158,10 @@
         <v>26</v>
       </c>
       <c r="G111" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H111" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I111" s="9">
         <v>46218</v>
@@ -8209,10 +8211,10 @@
         <v>26</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I112" s="5">
         <v>46218</v>
@@ -8262,10 +8264,10 @@
         <v>26</v>
       </c>
       <c r="G113" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H113" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I113" s="9">
         <v>46218</v>
@@ -8315,10 +8317,10 @@
         <v>26</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H114" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I114" s="5">
         <v>46218</v>
@@ -8368,10 +8370,10 @@
         <v>26</v>
       </c>
       <c r="G115" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H115" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I115" s="9">
         <v>46218</v>
@@ -8421,10 +8423,10 @@
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I116" s="5">
         <v>46218</v>
@@ -8474,10 +8476,10 @@
         <v>26</v>
       </c>
       <c r="G117" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H117" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I117" s="9">
         <v>46218</v>
@@ -8527,10 +8529,10 @@
         <v>26</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I118" s="5">
         <v>46218</v>
@@ -8580,10 +8582,10 @@
         <v>26</v>
       </c>
       <c r="G119" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H119" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I119" s="9">
         <v>46218</v>
@@ -8633,10 +8635,10 @@
         <v>26</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I120" s="5">
         <v>46219</v>
@@ -8675,7 +8677,7 @@
         <v>0</v>
       </c>
       <c r="U120" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
@@ -8696,10 +8698,10 @@
         <v>26</v>
       </c>
       <c r="G121" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H121" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I121" s="9">
         <v>46219</v>
@@ -8749,10 +8751,10 @@
         <v>26</v>
       </c>
       <c r="G122" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H122" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I122" s="5">
         <v>46219</v>
@@ -8802,10 +8804,10 @@
         <v>26</v>
       </c>
       <c r="G123" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H123" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I123" s="9">
         <v>46219</v>
@@ -8855,10 +8857,10 @@
         <v>26</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H124" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I124" s="5">
         <v>46219</v>
@@ -8908,10 +8910,10 @@
         <v>26</v>
       </c>
       <c r="G125" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H125" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I125" s="9">
         <v>46219</v>
@@ -8961,10 +8963,10 @@
         <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I126" s="5">
         <v>46219</v>
@@ -9014,10 +9016,10 @@
         <v>26</v>
       </c>
       <c r="G127" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H127" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I127" s="9">
         <v>46219</v>
@@ -9067,10 +9069,10 @@
         <v>26</v>
       </c>
       <c r="G128" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H128" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I128" s="5">
         <v>46219</v>
@@ -9120,10 +9122,10 @@
         <v>26</v>
       </c>
       <c r="G129" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H129" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I129" s="9">
         <v>46219</v>
@@ -9173,10 +9175,10 @@
         <v>26</v>
       </c>
       <c r="G130" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H130" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I130" s="5">
         <v>46219</v>
@@ -9226,10 +9228,10 @@
         <v>26</v>
       </c>
       <c r="G131" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H131" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I131" s="9">
         <v>46220</v>
@@ -9268,7 +9270,7 @@
         <v>0</v>
       </c>
       <c r="U131" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
@@ -9289,10 +9291,10 @@
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H132" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I132" s="5">
         <v>46220</v>
@@ -9342,10 +9344,10 @@
         <v>26</v>
       </c>
       <c r="G133" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H133" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I133" s="9">
         <v>46220</v>
@@ -9395,10 +9397,10 @@
         <v>26</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I134" s="5">
         <v>46220</v>
@@ -9448,10 +9450,10 @@
         <v>26</v>
       </c>
       <c r="G135" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H135" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I135" s="9">
         <v>46220</v>
@@ -9501,10 +9503,10 @@
         <v>26</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H136" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I136" s="5">
         <v>46220</v>
@@ -9554,10 +9556,10 @@
         <v>26</v>
       </c>
       <c r="G137" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H137" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I137" s="9">
         <v>46220</v>
@@ -9607,10 +9609,10 @@
         <v>26</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H138" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I138" s="5">
         <v>46220</v>
@@ -9660,10 +9662,10 @@
         <v>26</v>
       </c>
       <c r="G139" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H139" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I139" s="9">
         <v>46220</v>
@@ -9713,10 +9715,10 @@
         <v>26</v>
       </c>
       <c r="G140" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H140" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I140" s="5">
         <v>46220</v>
@@ -9766,10 +9768,10 @@
         <v>26</v>
       </c>
       <c r="G141" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H141" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I141" s="9">
         <v>46220</v>
@@ -9819,10 +9821,10 @@
         <v>26</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H142" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I142" s="5">
         <v>46223</v>
@@ -9861,7 +9863,7 @@
         <v>0</v>
       </c>
       <c r="U142" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -9882,10 +9884,10 @@
         <v>26</v>
       </c>
       <c r="G143" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H143" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I143" s="9">
         <v>46223</v>
@@ -9935,10 +9937,10 @@
         <v>26</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H144" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I144" s="5">
         <v>46223</v>
@@ -9988,10 +9990,10 @@
         <v>26</v>
       </c>
       <c r="G145" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H145" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I145" s="9">
         <v>46223</v>
@@ -10041,10 +10043,10 @@
         <v>26</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H146" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I146" s="5">
         <v>46223</v>
@@ -10094,10 +10096,10 @@
         <v>26</v>
       </c>
       <c r="G147" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H147" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I147" s="9">
         <v>46223</v>
@@ -10147,10 +10149,10 @@
         <v>26</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H148" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I148" s="5">
         <v>46223</v>
@@ -10200,10 +10202,10 @@
         <v>26</v>
       </c>
       <c r="G149" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H149" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I149" s="9">
         <v>46223</v>
@@ -10253,10 +10255,10 @@
         <v>26</v>
       </c>
       <c r="G150" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H150" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I150" s="5">
         <v>46223</v>
@@ -10306,10 +10308,10 @@
         <v>26</v>
       </c>
       <c r="G151" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H151" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I151" s="9">
         <v>46223</v>
@@ -10359,10 +10361,10 @@
         <v>26</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H152" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I152" s="5">
         <v>46223</v>
@@ -10412,10 +10414,10 @@
         <v>26</v>
       </c>
       <c r="G153" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H153" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I153" s="9">
         <v>46224</v>
@@ -10454,7 +10456,7 @@
         <v>0</v>
       </c>
       <c r="U153" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.25">
@@ -10475,10 +10477,10 @@
         <v>26</v>
       </c>
       <c r="G154" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H154" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I154" s="5">
         <v>46224</v>
@@ -10528,10 +10530,10 @@
         <v>26</v>
       </c>
       <c r="G155" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H155" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I155" s="9">
         <v>46224</v>
@@ -10581,10 +10583,10 @@
         <v>26</v>
       </c>
       <c r="G156" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H156" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I156" s="5">
         <v>46224</v>
@@ -10634,10 +10636,10 @@
         <v>26</v>
       </c>
       <c r="G157" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H157" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I157" s="9">
         <v>46224</v>
@@ -10687,10 +10689,10 @@
         <v>26</v>
       </c>
       <c r="G158" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H158" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I158" s="5">
         <v>46224</v>
@@ -10740,10 +10742,10 @@
         <v>26</v>
       </c>
       <c r="G159" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H159" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I159" s="9">
         <v>46224</v>
@@ -10793,10 +10795,10 @@
         <v>26</v>
       </c>
       <c r="G160" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H160" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I160" s="5">
         <v>46224</v>
@@ -10846,10 +10848,10 @@
         <v>26</v>
       </c>
       <c r="G161" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H161" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I161" s="9">
         <v>46224</v>
@@ -10899,10 +10901,10 @@
         <v>26</v>
       </c>
       <c r="G162" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H162" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I162" s="5">
         <v>46224</v>
@@ -10952,10 +10954,10 @@
         <v>26</v>
       </c>
       <c r="G163" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H163" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I163" s="9">
         <v>46224</v>
@@ -11005,10 +11007,10 @@
         <v>26</v>
       </c>
       <c r="G164" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H164" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I164" s="5">
         <v>46226</v>
@@ -11047,7 +11049,7 @@
         <v>0</v>
       </c>
       <c r="U164" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="165" spans="1:21" x14ac:dyDescent="0.25">
@@ -11068,10 +11070,10 @@
         <v>26</v>
       </c>
       <c r="G165" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H165" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I165" s="10"/>
       <c r="J165" s="9">
@@ -11119,10 +11121,10 @@
         <v>26</v>
       </c>
       <c r="G166" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H166" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I166" s="6"/>
       <c r="J166" s="5">
@@ -11170,10 +11172,10 @@
         <v>26</v>
       </c>
       <c r="G167" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H167" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I167" s="10"/>
       <c r="J167" s="9">
@@ -11221,10 +11223,10 @@
         <v>26</v>
       </c>
       <c r="G168" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H168" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I168" s="6"/>
       <c r="J168" s="5">
@@ -11272,10 +11274,10 @@
         <v>26</v>
       </c>
       <c r="G169" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H169" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I169" s="10"/>
       <c r="J169" s="9">
@@ -11323,10 +11325,10 @@
         <v>26</v>
       </c>
       <c r="G170" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H170" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I170" s="6"/>
       <c r="J170" s="5">
@@ -11374,10 +11376,10 @@
         <v>26</v>
       </c>
       <c r="G171" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H171" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I171" s="10"/>
       <c r="J171" s="9">
@@ -11425,10 +11427,10 @@
         <v>26</v>
       </c>
       <c r="G172" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H172" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I172" s="6"/>
       <c r="J172" s="5">
@@ -11476,10 +11478,10 @@
         <v>26</v>
       </c>
       <c r="G173" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H173" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I173" s="10"/>
       <c r="J173" s="9">
@@ -11527,10 +11529,10 @@
         <v>26</v>
       </c>
       <c r="G174" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H174" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I174" s="6"/>
       <c r="J174" s="5">
@@ -11667,7 +11669,7 @@
         <v>0</v>
       </c>
       <c r="U176" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="177" spans="1:21" x14ac:dyDescent="0.25">
@@ -12218,10 +12220,10 @@
         <v>26</v>
       </c>
       <c r="G187" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H187" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I187" s="9">
         <v>46230</v>
@@ -12260,7 +12262,7 @@
         <v>0</v>
       </c>
       <c r="U187" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="188" spans="1:21" x14ac:dyDescent="0.25">
@@ -12281,10 +12283,10 @@
         <v>26</v>
       </c>
       <c r="G188" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H188" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I188" s="5">
         <v>46230</v>
@@ -12334,10 +12336,10 @@
         <v>26</v>
       </c>
       <c r="G189" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H189" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I189" s="9">
         <v>46230</v>
@@ -12387,10 +12389,10 @@
         <v>26</v>
       </c>
       <c r="G190" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H190" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I190" s="5">
         <v>46230</v>
@@ -12440,10 +12442,10 @@
         <v>26</v>
       </c>
       <c r="G191" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H191" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I191" s="9">
         <v>46230</v>
@@ -12493,10 +12495,10 @@
         <v>26</v>
       </c>
       <c r="G192" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H192" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I192" s="5">
         <v>46230</v>
@@ -12546,10 +12548,10 @@
         <v>26</v>
       </c>
       <c r="G193" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H193" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I193" s="9">
         <v>46230</v>
@@ -12599,10 +12601,10 @@
         <v>26</v>
       </c>
       <c r="G194" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H194" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I194" s="5">
         <v>46230</v>
@@ -12652,10 +12654,10 @@
         <v>26</v>
       </c>
       <c r="G195" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H195" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I195" s="9">
         <v>46230</v>
@@ -12705,10 +12707,10 @@
         <v>26</v>
       </c>
       <c r="G196" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H196" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I196" s="5">
         <v>46230</v>
@@ -12758,10 +12760,10 @@
         <v>26</v>
       </c>
       <c r="G197" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H197" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I197" s="9">
         <v>46230</v>
@@ -12853,7 +12855,7 @@
         <v>0</v>
       </c>
       <c r="U198" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="199" spans="1:21" x14ac:dyDescent="0.25">
@@ -13446,7 +13448,7 @@
         <v>0</v>
       </c>
       <c r="U209" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="210" spans="1:21" x14ac:dyDescent="0.25">
@@ -14086,7 +14088,7 @@
         <v>0</v>
       </c>
       <c r="U221" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="222" spans="1:21" x14ac:dyDescent="0.25">
@@ -14149,7 +14151,7 @@
         <v>0</v>
       </c>
       <c r="U222" s="11" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Curva S actualizada 2026-09-06 13:14 Chile
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4327.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4327.xlsx
@@ -3290,7 +3290,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46213.54066168981</v>
+        <v>46271.64556232639</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -8872,7 +8872,7 @@
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46249.04035597222</v>
+        <v>46271.64561790509</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>224</v>

</xml_diff>